<commit_message>
Add Fabric F2 resources to cost calculator (XLSX + HTML)
- Fabric F2 capacity: 2 CUs × $0.19/CU/hr = $0.38/hr (indonesiacentral)
- Included items: Mirrored DB, SQL Endpoint, Semantic Model, Power BI Report
- XLSX: new 'Fabric Resources' sheet with architecture detail
- HTML: Fabric ON/OFF slider toggle
- 8hr total with Fabric: ~$11.72 (was ~$8.68 without)
</commit_message>
<xml_diff>
--- a/cost-calculator-8hr.xlsx
+++ b/cost-calculator-8hr.xlsx
@@ -10,6 +10,7 @@
     <sheet name="Resource Pricing" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="8-Hour Lab Simulation" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Hourly Breakdown" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Fabric Resources" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -18,11 +19,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="$#,##0.000000"/>
     <numFmt numFmtId="165" formatCode="$#,##0.00"/>
+    <numFmt numFmtId="166" formatCode="$#,##0.0000"/>
   </numFmts>
-  <fonts count="11">
+  <fonts count="14">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -66,6 +68,16 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="12"/>
     </font>
@@ -78,15 +90,20 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <sz val="10"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Consolas"/>
+      <sz val="9"/>
     </font>
     <font>
       <name val="Arial"/>
-      <b val="1"/>
-      <sz val="11"/>
+      <i val="1"/>
+      <color rgb="00C00000"/>
+      <sz val="9"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -101,6 +118,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2EFDA"/>
       </patternFill>
     </fill>
     <fill>
@@ -127,7 +149,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -143,13 +165,23 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="7" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="9" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="9" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="7" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -515,17 +547,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H12"/>
+  <dimension ref="A1:H18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="1" max="1"/>
     <col width="28" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
     <col width="18" customWidth="1" min="7" max="7"/>
-    <col width="28" customWidth="1" min="8" max="8"/>
+    <col width="30" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -763,120 +795,126 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>GPT-5 Input</t>
+          <t>Fabric Capacity</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>GlobalStandard cap-20</t>
+          <t>F2 (2 CUs)</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>eastus2</t>
+          <t>indonesiacentral</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Per Token</t>
+          <t>Provisioned</t>
         </is>
       </c>
       <c r="E7" s="3" t="n">
-        <v>0.0025</v>
+        <v>0.38</v>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>1K tokens</t>
-        </is>
-      </c>
-      <c r="G7" s="3" t="n"/>
+          <t>1 Hour</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="n">
+        <v>0.38</v>
+      </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>Est. gpt-4o rate proxy</t>
+          <t>2 CUs × $0.19/CU/hr</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>GPT-5 Output</t>
+          <t>Fabric - Mirrored DB</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>GlobalStandard cap-20</t>
+          <t>Mirroring (within F2)</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>eastus2</t>
+          <t>indonesiacentral</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Per Token</t>
+          <t>Included in F2</t>
         </is>
       </c>
       <c r="E8" s="3" t="n">
-        <v>0.01</v>
+        <v>0</v>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>1K tokens</t>
-        </is>
-      </c>
-      <c r="G8" s="3" t="n"/>
+          <t>CU consumption</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>Est. gpt-4o rate proxy</t>
+          <t>Consumes CUs from F2 capacity</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>text-embedding-3-small</t>
+          <t>Fabric - SQL Endpoint</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>GlobalStandard cap-50</t>
+          <t>SQL Analytics Endpoint</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>eastus2</t>
+          <t>indonesiacentral</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Per Token</t>
+          <t>Included in F2</t>
         </is>
       </c>
       <c r="E9" s="3" t="n">
-        <v>2.5e-05</v>
+        <v>0</v>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>1K tokens</t>
-        </is>
-      </c>
-      <c r="G9" s="3" t="n"/>
+          <t>CU consumption</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>Confirmed from API</t>
+          <t>Consumes CUs from F2 capacity</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>VNet</t>
+          <t>Fabric - Semantic Model</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>vnet-lab513-2139d8</t>
+          <t>Direct Lake on SQL</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -886,7 +924,7 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Free</t>
+          <t>Included in F2</t>
         </is>
       </c>
       <c r="E10" s="3" t="n">
@@ -894,7 +932,7 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>CU consumption</t>
         </is>
       </c>
       <c r="G10" s="3" t="n">
@@ -902,19 +940,19 @@
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>No charge</t>
+          <t>Consumes CUs from F2 capacity</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>NSG</t>
+          <t>Fabric - Power BI Report</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>nsg-lab513-2139d8</t>
+          <t>FAQ_rpt</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -924,7 +962,7 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Free</t>
+          <t>Included in F2</t>
         </is>
       </c>
       <c r="E11" s="3" t="n">
@@ -932,7 +970,7 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>CU consumption</t>
         </is>
       </c>
       <c r="G11" s="3" t="n">
@@ -940,43 +978,265 @@
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>No charge</t>
+          <t>Consumes CUs from F2 capacity</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
+          <t>GPT-5 Input</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>GlobalStandard cap-20</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>eastus2</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Per Token</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="n">
+        <v>0.0025</v>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>1K tokens</t>
+        </is>
+      </c>
+      <c r="G12" s="3" t="n"/>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>Est. gpt-4o rate proxy</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>GPT-5 Output</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>GlobalStandard cap-20</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>eastus2</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>Per Token</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>1K tokens</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="n"/>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>Est. gpt-4o rate proxy</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>text-embedding-3-small</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>GlobalStandard cap-50</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>eastus2</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Per Token</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="n">
+        <v>2.5e-05</v>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>1K tokens</t>
+        </is>
+      </c>
+      <c r="G14" s="3" t="n"/>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>Confirmed from API</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>AI Services Account</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>S0</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>eastus2</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="G15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>No base charge</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>VNet</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>vnet-lab513-2139d8</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>indonesiacentral</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G16" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>No charge</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>NSG</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>nsg-lab513-2139d8</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>indonesiacentral</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G17" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>No charge</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
           <t>AI Foundry Project</t>
         </is>
       </c>
-      <c r="B12" s="2" t="inlineStr">
+      <c r="B18" s="2" t="inlineStr">
         <is>
           <t>FAQ-Assistant-project</t>
         </is>
       </c>
-      <c r="C12" s="2" t="inlineStr">
+      <c r="C18" s="2" t="inlineStr">
         <is>
           <t>eastus2</t>
         </is>
       </c>
-      <c r="D12" s="2" t="inlineStr">
+      <c r="D18" s="2" t="inlineStr">
         <is>
           <t>Free</t>
         </is>
       </c>
-      <c r="E12" s="3" t="n">
+      <c r="E18" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="F12" s="2" t="inlineStr">
+      <c r="F18" s="2" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="G12" s="3" t="n">
+      <c r="G18" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="H12" s="2" t="inlineStr">
+      <c r="H18" s="2" t="inlineStr">
         <is>
           <t>Included in AI Services</t>
         </is>
@@ -993,20 +1253,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E29"/>
+  <dimension ref="A1:E37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="32" customWidth="1" min="1" max="1"/>
+    <col width="38" customWidth="1" min="1" max="1"/>
     <col width="32" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="5" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Lab513 Cost Simulation - 8 Hour Workshop</t>
+          <t>Lab513 Cost Simulation - 8 Hour Workshop (incl. Fabric F2)</t>
         </is>
       </c>
     </row>
@@ -1149,195 +1409,284 @@
       </c>
       <c r="E11" s="8" t="inlineStr"/>
     </row>
-    <row r="13">
-      <c r="A13" s="5" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>Fabric F2 active</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="C12" s="6" t="inlineStr"/>
+      <c r="E12" s="8" t="inlineStr">
+        <is>
+          <t>F2 provisioned = always-on cost</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
         <is>
           <t>COST BREAKDOWN (8 Hours)</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="9" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="9" t="inlineStr">
         <is>
           <t>Component</t>
         </is>
       </c>
-      <c r="B14" s="9" t="inlineStr">
+      <c r="B15" s="9" t="inlineStr">
         <is>
           <t>Calculation</t>
         </is>
       </c>
-      <c r="C14" s="9" t="inlineStr">
+      <c r="C15" s="9" t="inlineStr">
         <is>
           <t>Cost (USD)</t>
         </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="6" t="inlineStr">
-        <is>
-          <t>VM Compute (D2s_v5 Windows)</t>
-        </is>
-      </c>
-      <c r="B15" s="6" t="inlineStr">
-        <is>
-          <t>8 hrs × $0.200/hr</t>
-        </is>
-      </c>
-      <c r="C15" s="10">
-        <f>B4*0.2</f>
-        <v/>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t>VM OS Disk (S10 128GB)</t>
+          <t>VM Compute (D2s_v5 Windows)</t>
         </is>
       </c>
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>8 hrs × $5.89/730/hr</t>
+          <t>8 hrs × $0.200/hr</t>
         </is>
       </c>
       <c r="C16" s="10">
-        <f>B4*(5.89/730)</f>
+        <f>B4*0.2</f>
         <v/>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="6" t="inlineStr">
         <is>
-          <t>SQL Compute (Serverless Gen5)</t>
+          <t>VM OS Disk (S10 128GB)</t>
         </is>
       </c>
       <c r="B17" s="6" t="inlineStr">
         <is>
-          <t>8 hrs × vCores × $0.6849/vCore/hr</t>
+          <t>8 hrs × $5.89/730/hr</t>
         </is>
       </c>
       <c r="C17" s="10">
-        <f>B4*B5*0.6849</f>
+        <f>B4*(5.89/730)</f>
         <v/>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t>SQL Storage (Hyperscale)</t>
+          <t>SQL Compute (Serverless Gen5)</t>
         </is>
       </c>
       <c r="B18" s="6" t="inlineStr">
         <is>
-          <t>GB × $0.108/mo prorated</t>
+          <t>8 hrs × vCores × $0.6849/vCore/hr</t>
         </is>
       </c>
       <c r="C18" s="10">
-        <f>B6*0.108*(B4/730)</f>
+        <f>B4*B5*0.6849</f>
         <v/>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
         <is>
-          <t>GPT-5 Input Tokens</t>
+          <t>SQL Storage (Hyperscale)</t>
         </is>
       </c>
       <c r="B19" s="6" t="inlineStr">
         <is>
-          <t>chats × tokens × $0.0025/1K</t>
+          <t>GB × $0.108/mo prorated</t>
         </is>
       </c>
       <c r="C19" s="10">
-        <f>B7*B8/1000*0.0025</f>
+        <f>B6*0.108*(B4/730)</f>
         <v/>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="6" t="inlineStr">
-        <is>
-          <t>GPT-5 Output Tokens</t>
-        </is>
-      </c>
-      <c r="B20" s="6" t="inlineStr">
-        <is>
-          <t>chats × tokens × $0.01/1K</t>
-        </is>
-      </c>
-      <c r="C20" s="10">
-        <f>B7*B9/1000*0.01</f>
+      <c r="A20" s="11" t="inlineStr">
+        <is>
+          <t>Microsoft Fabric F2 Capacity</t>
+        </is>
+      </c>
+      <c r="B20" s="12" t="inlineStr">
+        <is>
+          <t>8 hrs × $0.38/hr (2 CUs)</t>
+        </is>
+      </c>
+      <c r="C20" s="13">
+        <f>B4*0.38</f>
         <v/>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="6" t="inlineStr">
-        <is>
-          <t>Embedding Tokens</t>
-        </is>
-      </c>
-      <c r="B21" s="6" t="inlineStr">
-        <is>
-          <t>calls × tokens × $0.000025/1K</t>
-        </is>
-      </c>
-      <c r="C21" s="10">
-        <f>B10*B11/1000*0.000025</f>
-        <v/>
+      <c r="A21" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  └ Mirrored DB + Endpoint + Model + Report</t>
+        </is>
+      </c>
+      <c r="B21" s="14" t="inlineStr">
+        <is>
+          <t>Included in F2 capacity</t>
+        </is>
+      </c>
+      <c r="C21" s="13" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="6" t="inlineStr">
         <is>
+          <t>GPT-5 Input Tokens</t>
+        </is>
+      </c>
+      <c r="B22" s="6" t="inlineStr">
+        <is>
+          <t>chats × tokens × $0.0025/1K</t>
+        </is>
+      </c>
+      <c r="C22" s="10">
+        <f>B7*B8/1000*0.0025</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="6" t="inlineStr">
+        <is>
+          <t>GPT-5 Output Tokens</t>
+        </is>
+      </c>
+      <c r="B23" s="6" t="inlineStr">
+        <is>
+          <t>chats × tokens × $0.01/1K</t>
+        </is>
+      </c>
+      <c r="C23" s="10">
+        <f>B7*B9/1000*0.01</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="6" t="inlineStr">
+        <is>
+          <t>Embedding Tokens</t>
+        </is>
+      </c>
+      <c r="B24" s="6" t="inlineStr">
+        <is>
+          <t>calls × tokens × $0.000025/1K</t>
+        </is>
+      </c>
+      <c r="C24" s="10">
+        <f>B10*B11/1000*0.000025</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="6" t="inlineStr">
+        <is>
           <t>VNet + NSG + AI Project</t>
         </is>
       </c>
-      <c r="B22" s="6" t="inlineStr">
+      <c r="B25" s="6" t="inlineStr">
         <is>
           <t>Free</t>
         </is>
       </c>
-      <c r="C22" s="10" t="n">
+      <c r="C25" s="10" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="11" t="inlineStr">
+    <row r="27">
+      <c r="A27" s="15" t="inlineStr">
         <is>
           <t>TOTAL COST (8 HOURS)</t>
         </is>
       </c>
-      <c r="B24" s="12" t="n"/>
-      <c r="C24" s="13">
-        <f>SUM(C15:C22)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="5" t="inlineStr">
+      <c r="B27" s="16" t="n"/>
+      <c r="C27" s="17">
+        <f>SUM(C16:C25)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
         <is>
           <t>Average cost per hour</t>
         </is>
       </c>
-      <c r="C26" s="10">
-        <f>C24/B4</f>
-        <v/>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="6" t="inlineStr">
+      <c r="C29" s="10">
+        <f>C27/B4</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="6" t="inlineStr">
         <is>
           <t>Monthly projection (if always-on 730hrs)</t>
         </is>
       </c>
-      <c r="C27" s="10">
-        <f>C26*730</f>
-        <v/>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="14" t="inlineStr">
-        <is>
-          <t>TIP: Deallocate VM when not in use to save $0.20/hr ($146/month)</t>
+      <c r="C30" s="10">
+        <f>C29*730</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>COST DISTRIBUTION</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Infrastructure (VM+Disk+SQL)</t>
+        </is>
+      </c>
+      <c r="C33" s="18">
+        <f>C16+C17+C18+C19</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="19" t="inlineStr">
+        <is>
+          <t>Microsoft Fabric (F2)</t>
+        </is>
+      </c>
+      <c r="C34" s="20">
+        <f>C20</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>AI Tokens (GPT-5 + Embed)</t>
+        </is>
+      </c>
+      <c r="C35" s="18">
+        <f>C22+C23+C24</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="21" t="inlineStr">
+        <is>
+          <t>TIP: Pause Fabric capacity &amp; deallocate VM when not in use to save $0.58/hr</t>
         </is>
       </c>
     </row>
@@ -1355,21 +1704,22 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F12"/>
+  <dimension ref="A1:G12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Hour-by-Hour Cost Accumulation</t>
+          <t>Hour-by-Hour Cost Accumulation (with Fabric F2)</t>
         </is>
       </c>
     </row>
@@ -1396,10 +1746,15 @@
       </c>
       <c r="E3" s="9" t="inlineStr">
         <is>
+          <t>Fabric F2 ($)</t>
+        </is>
+      </c>
+      <c r="F3" s="9" t="inlineStr">
+        <is>
           <t>AI Tokens ($)</t>
         </is>
       </c>
-      <c r="F3" s="9" t="inlineStr">
+      <c r="G3" s="9" t="inlineStr">
         <is>
           <t>Running Total ($)</t>
         </is>
@@ -1409,22 +1764,25 @@
       <c r="A4" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="B4" s="15" t="n">
+      <c r="B4" s="10" t="n">
         <v>0.2</v>
       </c>
-      <c r="C4" s="10">
+      <c r="C4" s="22">
         <f>5.89/730</f>
         <v/>
       </c>
-      <c r="D4" s="15" t="n">
+      <c r="D4" s="10" t="n">
         <v>0.6849</v>
       </c>
-      <c r="E4" s="10">
+      <c r="E4" s="13" t="n">
+        <v>0.38</v>
+      </c>
+      <c r="F4" s="22">
         <f>(50*500/1000*0.0025 + 50*300/1000*0.01 + 100*200/1000*0.000025)/8</f>
         <v/>
       </c>
-      <c r="F4" s="16">
-        <f>B4+C4+D4+E4</f>
+      <c r="G4" s="23">
+        <f>B4+C4+D4+E4+F4</f>
         <v/>
       </c>
     </row>
@@ -1432,22 +1790,25 @@
       <c r="A5" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="B5" s="15" t="n">
+      <c r="B5" s="10" t="n">
         <v>0.2</v>
       </c>
-      <c r="C5" s="10">
+      <c r="C5" s="22">
         <f>5.89/730</f>
         <v/>
       </c>
-      <c r="D5" s="15" t="n">
+      <c r="D5" s="10" t="n">
         <v>0.6849</v>
       </c>
-      <c r="E5" s="10">
+      <c r="E5" s="13" t="n">
+        <v>0.38</v>
+      </c>
+      <c r="F5" s="22">
         <f>(50*500/1000*0.0025 + 50*300/1000*0.01 + 100*200/1000*0.000025)/8</f>
         <v/>
       </c>
-      <c r="F5" s="16">
-        <f>F4+B5+C5+D5+E5</f>
+      <c r="G5" s="23">
+        <f>G4+B5+C5+D5+E5+F5</f>
         <v/>
       </c>
     </row>
@@ -1455,22 +1816,25 @@
       <c r="A6" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="B6" s="15" t="n">
+      <c r="B6" s="10" t="n">
         <v>0.2</v>
       </c>
-      <c r="C6" s="10">
+      <c r="C6" s="22">
         <f>5.89/730</f>
         <v/>
       </c>
-      <c r="D6" s="15" t="n">
+      <c r="D6" s="10" t="n">
         <v>0.6849</v>
       </c>
-      <c r="E6" s="10">
+      <c r="E6" s="13" t="n">
+        <v>0.38</v>
+      </c>
+      <c r="F6" s="22">
         <f>(50*500/1000*0.0025 + 50*300/1000*0.01 + 100*200/1000*0.000025)/8</f>
         <v/>
       </c>
-      <c r="F6" s="16">
-        <f>F5+B6+C6+D6+E6</f>
+      <c r="G6" s="23">
+        <f>G5+B6+C6+D6+E6+F6</f>
         <v/>
       </c>
     </row>
@@ -1478,22 +1842,25 @@
       <c r="A7" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="B7" s="15" t="n">
+      <c r="B7" s="10" t="n">
         <v>0.2</v>
       </c>
-      <c r="C7" s="10">
+      <c r="C7" s="22">
         <f>5.89/730</f>
         <v/>
       </c>
-      <c r="D7" s="15" t="n">
+      <c r="D7" s="10" t="n">
         <v>0.6849</v>
       </c>
-      <c r="E7" s="10">
+      <c r="E7" s="13" t="n">
+        <v>0.38</v>
+      </c>
+      <c r="F7" s="22">
         <f>(50*500/1000*0.0025 + 50*300/1000*0.01 + 100*200/1000*0.000025)/8</f>
         <v/>
       </c>
-      <c r="F7" s="16">
-        <f>F6+B7+C7+D7+E7</f>
+      <c r="G7" s="23">
+        <f>G6+B7+C7+D7+E7+F7</f>
         <v/>
       </c>
     </row>
@@ -1501,22 +1868,25 @@
       <c r="A8" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="B8" s="15" t="n">
+      <c r="B8" s="10" t="n">
         <v>0.2</v>
       </c>
-      <c r="C8" s="10">
+      <c r="C8" s="22">
         <f>5.89/730</f>
         <v/>
       </c>
-      <c r="D8" s="15" t="n">
+      <c r="D8" s="10" t="n">
         <v>0.6849</v>
       </c>
-      <c r="E8" s="10">
+      <c r="E8" s="13" t="n">
+        <v>0.38</v>
+      </c>
+      <c r="F8" s="22">
         <f>(50*500/1000*0.0025 + 50*300/1000*0.01 + 100*200/1000*0.000025)/8</f>
         <v/>
       </c>
-      <c r="F8" s="16">
-        <f>F7+B8+C8+D8+E8</f>
+      <c r="G8" s="23">
+        <f>G7+B8+C8+D8+E8+F8</f>
         <v/>
       </c>
     </row>
@@ -1524,22 +1894,25 @@
       <c r="A9" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="B9" s="15" t="n">
+      <c r="B9" s="10" t="n">
         <v>0.2</v>
       </c>
-      <c r="C9" s="10">
+      <c r="C9" s="22">
         <f>5.89/730</f>
         <v/>
       </c>
-      <c r="D9" s="15" t="n">
+      <c r="D9" s="10" t="n">
         <v>0.6849</v>
       </c>
-      <c r="E9" s="10">
+      <c r="E9" s="13" t="n">
+        <v>0.38</v>
+      </c>
+      <c r="F9" s="22">
         <f>(50*500/1000*0.0025 + 50*300/1000*0.01 + 100*200/1000*0.000025)/8</f>
         <v/>
       </c>
-      <c r="F9" s="16">
-        <f>F8+B9+C9+D9+E9</f>
+      <c r="G9" s="23">
+        <f>G8+B9+C9+D9+E9+F9</f>
         <v/>
       </c>
     </row>
@@ -1547,22 +1920,25 @@
       <c r="A10" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="B10" s="15" t="n">
+      <c r="B10" s="10" t="n">
         <v>0.2</v>
       </c>
-      <c r="C10" s="10">
+      <c r="C10" s="22">
         <f>5.89/730</f>
         <v/>
       </c>
-      <c r="D10" s="15" t="n">
+      <c r="D10" s="10" t="n">
         <v>0.6849</v>
       </c>
-      <c r="E10" s="10">
+      <c r="E10" s="13" t="n">
+        <v>0.38</v>
+      </c>
+      <c r="F10" s="22">
         <f>(50*500/1000*0.0025 + 50*300/1000*0.01 + 100*200/1000*0.000025)/8</f>
         <v/>
       </c>
-      <c r="F10" s="16">
-        <f>F9+B10+C10+D10+E10</f>
+      <c r="G10" s="23">
+        <f>G9+B10+C10+D10+E10+F10</f>
         <v/>
       </c>
     </row>
@@ -1570,39 +1946,304 @@
       <c r="A11" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="B11" s="15" t="n">
+      <c r="B11" s="10" t="n">
         <v>0.2</v>
       </c>
-      <c r="C11" s="10">
+      <c r="C11" s="22">
         <f>5.89/730</f>
         <v/>
       </c>
-      <c r="D11" s="15" t="n">
+      <c r="D11" s="10" t="n">
         <v>0.6849</v>
       </c>
-      <c r="E11" s="10">
+      <c r="E11" s="13" t="n">
+        <v>0.38</v>
+      </c>
+      <c r="F11" s="22">
         <f>(50*500/1000*0.0025 + 50*300/1000*0.01 + 100*200/1000*0.000025)/8</f>
         <v/>
       </c>
-      <c r="F11" s="16">
-        <f>F10+B11+C11+D11+E11</f>
+      <c r="G11" s="23">
+        <f>G10+B11+C11+D11+E11+F11</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="17" t="inlineStr">
+      <c r="A12" s="24" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="F12" s="13">
-        <f>F11</f>
+      <c r="G12" s="17">
+        <f>G11</f>
         <v/>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A1:G1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D22"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="36" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Microsoft Fabric Resources (Lab Exercise 5)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>Fabric Capacity SKU</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>F2 (2 Capacity Units)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Region</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>indonesiacentral</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>CU Rate</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>$0.19/CU/hour</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>F2 Hourly Cost</t>
+        </is>
+      </c>
+      <c r="B6" s="18">
+        <f>2*0.19</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>F2 Monthly Cost (730hr)</t>
+        </is>
+      </c>
+      <c r="B7" s="18">
+        <f>B6*730</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>FABRIC ITEMS IN LAB</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="25" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B10" s="25" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="C10" s="25" t="inlineStr">
+        <is>
+          <t>CU Consumption</t>
+        </is>
+      </c>
+      <c r="D10" s="25" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Workspace2139d8</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Workspace</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Container only</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>Named per LAB_INSTANCE_ID</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>faq-ai-assistant-db</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Mirrored Azure SQL DB</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Data Movement CUs</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Mirrors dbo.FAQ_Content to OneLake</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>SQL Analytics Endpoint</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Auto-created endpoint</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Data Warehouse CUs</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>Query mirrored Delta tables</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>FAQ_Content</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Semantic Model (Direct Lake)</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Power BI CUs</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Storage mode: Direct Lake on SQL</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>FAQ_rpt</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Power BI Report</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Power BI CUs</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>Created via Copilot in Fabric</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>ARCHITECTURE</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="26" t="inlineStr">
+        <is>
+          <t>Azure SQL Hyperscale → Fabric Mirroring → OneLake (Delta) → SQL Endpoint → Semantic Model → Power BI</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="8" t="inlineStr">
+        <is>
+          <t>NOTE: All Fabric workloads consume CUs from the provisioned F2 capacity.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="8" t="inlineStr">
+        <is>
+          <t>No additional per-item cost beyond the F2 base rate of $0.38/hr.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="27" t="inlineStr">
+        <is>
+          <t>Pause capacity when not in use to stop billing.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:D1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Regenerate XLSX with Region column and disclaimer
</commit_message>
<xml_diff>
--- a/cost-calculator-8hr.xlsx
+++ b/cost-calculator-8hr.xlsx
@@ -24,7 +24,7 @@
     <numFmt numFmtId="165" formatCode="$#,##0.00"/>
     <numFmt numFmtId="166" formatCode="$#,##0.0000"/>
   </numFmts>
-  <fonts count="14">
+  <fonts count="16">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -67,12 +67,7 @@
     </font>
     <font>
       <name val="Arial"/>
-      <b val="1"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <i val="1"/>
+      <color rgb="00666666"/>
       <sz val="9"/>
     </font>
     <font>
@@ -83,9 +78,27 @@
     </font>
     <font>
       <name val="Arial"/>
-      <i val="1"/>
+      <b val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
       <color rgb="00C00000"/>
       <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
     </font>
     <font>
       <name val="Arial"/>
@@ -94,12 +107,6 @@
     </font>
     <font>
       <name val="Consolas"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <i val="1"/>
-      <color rgb="00C00000"/>
       <sz val="9"/>
     </font>
   </fonts>
@@ -149,7 +156,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -161,27 +168,29 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="9" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="8" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="13" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="7" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -555,9 +564,9 @@
     <col width="18" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
     <col width="18" customWidth="1" min="7" max="7"/>
-    <col width="30" customWidth="1" min="8" max="8"/>
+    <col width="32" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -636,7 +645,7 @@
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>2 vCPU, 8GB RAM</t>
+          <t>INCL. Windows license; 2 vCPU 8GB</t>
         </is>
       </c>
     </row>
@@ -673,9 +682,10 @@
         <f>E3/730</f>
         <v/>
       </c>
-      <c r="H3" s="2">
-        <f>E3/730</f>
-        <v/>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>Standard_LRS; 127GB actual</t>
+        </is>
       </c>
     </row>
     <row r="4">
@@ -749,9 +759,10 @@
         <f>E5/730</f>
         <v/>
       </c>
-      <c r="H5" s="2">
-        <f>E5/730</f>
-        <v/>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>$0.108/GB/month</t>
+        </is>
       </c>
     </row>
     <row r="6">
@@ -787,9 +798,10 @@
         <f>E6/730</f>
         <v/>
       </c>
-      <c r="H6" s="2">
-        <f>E6/730</f>
-        <v/>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>$0.0864/GB/month</t>
+        </is>
       </c>
     </row>
     <row r="7">
@@ -826,7 +838,7 @@
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>2 CUs × $0.19/CU/hr</t>
+          <t>2 CUs x $0.19/CU/hr</t>
         </is>
       </c>
     </row>
@@ -864,7 +876,7 @@
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>Consumes CUs from F2 capacity</t>
+          <t>Consumes CUs from F2</t>
         </is>
       </c>
     </row>
@@ -902,7 +914,7 @@
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>Consumes CUs from F2 capacity</t>
+          <t>Consumes CUs from F2</t>
         </is>
       </c>
     </row>
@@ -940,7 +952,7 @@
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>Consumes CUs from F2 capacity</t>
+          <t>Consumes CUs from F2</t>
         </is>
       </c>
     </row>
@@ -978,7 +990,7 @@
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>Consumes CUs from F2 capacity</t>
+          <t>Consumes CUs from F2</t>
         </is>
       </c>
     </row>
@@ -1014,7 +1026,7 @@
       <c r="G12" s="3" t="n"/>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>Est. gpt-4o rate proxy</t>
+          <t>Est. gpt-4o-1120 rate</t>
         </is>
       </c>
     </row>
@@ -1050,7 +1062,7 @@
       <c r="G13" s="3" t="n"/>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>Est. gpt-4o rate proxy</t>
+          <t>Est. gpt-4o-1120 rate</t>
         </is>
       </c>
     </row>
@@ -1253,14 +1265,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E37"/>
+  <dimension ref="A1:F41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
-    <col width="32" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="5" customWidth="1" min="4" max="4"/>
-    <col width="30" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1423,276 +1435,365 @@
       <c r="C12" s="6" t="inlineStr"/>
       <c r="E12" s="8" t="inlineStr">
         <is>
-          <t>F2 provisioned = always-on cost</t>
+          <t>F2 provisioned = always-on</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="5" t="inlineStr">
+      <c r="A14" s="9" t="inlineStr">
         <is>
           <t>COST BREAKDOWN (8 Hours)</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="9" t="inlineStr">
+      <c r="A15" s="10" t="inlineStr">
         <is>
           <t>Component</t>
         </is>
       </c>
-      <c r="B15" s="9" t="inlineStr">
+      <c r="B15" s="10" t="inlineStr">
+        <is>
+          <t>Region</t>
+        </is>
+      </c>
+      <c r="C15" s="10" t="inlineStr">
         <is>
           <t>Calculation</t>
         </is>
       </c>
-      <c r="C15" s="9" t="inlineStr">
+      <c r="D15" s="10" t="inlineStr">
         <is>
           <t>Cost (USD)</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="6" t="inlineStr">
+      <c r="A16" s="2" t="inlineStr">
         <is>
           <t>VM Compute (D2s_v5 Windows)</t>
         </is>
       </c>
-      <c r="B16" s="6" t="inlineStr">
-        <is>
-          <t>8 hrs × $0.200/hr</t>
-        </is>
-      </c>
-      <c r="C16" s="10">
+      <c r="B16" s="11" t="inlineStr">
+        <is>
+          <t>indonesiacentral</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>8 hrs x $0.200/hr</t>
+        </is>
+      </c>
+      <c r="D16" s="12">
         <f>B4*0.2</f>
         <v/>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="6" t="inlineStr">
+      <c r="A17" s="2" t="inlineStr">
         <is>
           <t>VM OS Disk (S10 128GB)</t>
         </is>
       </c>
-      <c r="B17" s="6" t="inlineStr">
-        <is>
-          <t>8 hrs × $5.89/730/hr</t>
-        </is>
-      </c>
-      <c r="C17" s="10">
+      <c r="B17" s="11" t="inlineStr">
+        <is>
+          <t>indonesiacentral</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>8 hrs x $5.89/730/hr</t>
+        </is>
+      </c>
+      <c r="D17" s="12">
         <f>B4*(5.89/730)</f>
         <v/>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="6" t="inlineStr">
+      <c r="A18" s="2" t="inlineStr">
         <is>
           <t>SQL Compute (Serverless Gen5)</t>
         </is>
       </c>
-      <c r="B18" s="6" t="inlineStr">
-        <is>
-          <t>8 hrs × vCores × $0.6849/vCore/hr</t>
-        </is>
-      </c>
-      <c r="C18" s="10">
+      <c r="B18" s="11" t="inlineStr">
+        <is>
+          <t>indonesiacentral</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>8 hrs x vCores x $0.6849</t>
+        </is>
+      </c>
+      <c r="D18" s="12">
         <f>B4*B5*0.6849</f>
         <v/>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="6" t="inlineStr">
+      <c r="A19" s="2" t="inlineStr">
         <is>
           <t>SQL Storage (Hyperscale)</t>
         </is>
       </c>
-      <c r="B19" s="6" t="inlineStr">
-        <is>
-          <t>GB × $0.108/mo prorated</t>
-        </is>
-      </c>
-      <c r="C19" s="10">
+      <c r="B19" s="11" t="inlineStr">
+        <is>
+          <t>indonesiacentral</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>GB x $0.108/mo prorated</t>
+        </is>
+      </c>
+      <c r="D19" s="12">
         <f>B6*0.108*(B4/730)</f>
         <v/>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="11" t="inlineStr">
+      <c r="A20" s="13" t="inlineStr">
         <is>
           <t>Microsoft Fabric F2 Capacity</t>
         </is>
       </c>
-      <c r="B20" s="12" t="inlineStr">
-        <is>
-          <t>8 hrs × $0.38/hr (2 CUs)</t>
-        </is>
-      </c>
-      <c r="C20" s="13">
+      <c r="B20" s="14" t="inlineStr">
+        <is>
+          <t>indonesiacentral</t>
+        </is>
+      </c>
+      <c r="C20" s="13" t="inlineStr">
+        <is>
+          <t>8 hrs x $0.38/hr (2 CUs)</t>
+        </is>
+      </c>
+      <c r="D20" s="15">
         <f>B4*0.38</f>
         <v/>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="14" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  └ Mirrored DB + Endpoint + Model + Report</t>
-        </is>
-      </c>
-      <c r="B21" s="14" t="inlineStr">
-        <is>
-          <t>Included in F2 capacity</t>
-        </is>
-      </c>
-      <c r="C21" s="13" t="n">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  - Mirrored DB + Endpoint + Model + Report</t>
+        </is>
+      </c>
+      <c r="B21" s="11" t="inlineStr">
+        <is>
+          <t>indonesiacentral</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>Included in F2</t>
+        </is>
+      </c>
+      <c r="D21" s="12" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="6" t="inlineStr">
+      <c r="A22" s="2" t="inlineStr">
         <is>
           <t>GPT-5 Input Tokens</t>
         </is>
       </c>
-      <c r="B22" s="6" t="inlineStr">
-        <is>
-          <t>chats × tokens × $0.0025/1K</t>
-        </is>
-      </c>
-      <c r="C22" s="10">
+      <c r="B22" s="11" t="inlineStr">
+        <is>
+          <t>eastus2</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>chats x tokens x $0.0025/1K</t>
+        </is>
+      </c>
+      <c r="D22" s="12">
         <f>B7*B8/1000*0.0025</f>
         <v/>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="6" t="inlineStr">
+      <c r="A23" s="2" t="inlineStr">
         <is>
           <t>GPT-5 Output Tokens</t>
         </is>
       </c>
-      <c r="B23" s="6" t="inlineStr">
-        <is>
-          <t>chats × tokens × $0.01/1K</t>
-        </is>
-      </c>
-      <c r="C23" s="10">
+      <c r="B23" s="11" t="inlineStr">
+        <is>
+          <t>eastus2</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>chats x tokens x $0.01/1K</t>
+        </is>
+      </c>
+      <c r="D23" s="12">
         <f>B7*B9/1000*0.01</f>
         <v/>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="6" t="inlineStr">
+      <c r="A24" s="2" t="inlineStr">
         <is>
           <t>Embedding Tokens</t>
         </is>
       </c>
-      <c r="B24" s="6" t="inlineStr">
-        <is>
-          <t>calls × tokens × $0.000025/1K</t>
-        </is>
-      </c>
-      <c r="C24" s="10">
+      <c r="B24" s="11" t="inlineStr">
+        <is>
+          <t>eastus2</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>calls x tokens x $0.000025/1K</t>
+        </is>
+      </c>
+      <c r="D24" s="12">
         <f>B10*B11/1000*0.000025</f>
         <v/>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="6" t="inlineStr">
+      <c r="A25" s="2" t="inlineStr">
         <is>
           <t>VNet + NSG + AI Project</t>
         </is>
       </c>
-      <c r="B25" s="6" t="inlineStr">
+      <c r="B25" s="11" t="inlineStr">
+        <is>
+          <t>both</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
         <is>
           <t>Free</t>
         </is>
       </c>
-      <c r="C25" s="10" t="n">
+      <c r="D25" s="12" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="15" t="inlineStr">
+    <row r="26">
+      <c r="A26" s="16" t="inlineStr">
         <is>
           <t>TOTAL COST (8 HOURS)</t>
         </is>
       </c>
-      <c r="B27" s="16" t="n"/>
-      <c r="C27" s="17">
-        <f>SUM(C16:C25)</f>
-        <v/>
+      <c r="B26" s="17" t="n"/>
+      <c r="C26" s="17" t="n"/>
+      <c r="D26" s="18">
+        <f>SUM(D16:D25)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>HOW TO READ:</t>
+        </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="5" t="inlineStr">
-        <is>
-          <t>Average cost per hour</t>
-        </is>
-      </c>
-      <c r="C29" s="10">
-        <f>C27/B4</f>
-        <v/>
+      <c r="A29" s="6" t="inlineStr">
+        <is>
+          <t>Total Cost (above) = total biaya selama DURASI yang dipilih (8 jam)</t>
+        </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="6" t="inlineStr">
         <is>
-          <t>Monthly projection (if always-on 730hrs)</t>
-        </is>
-      </c>
-      <c r="C30" s="10">
-        <f>C29*730</f>
-        <v/>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="5" t="inlineStr">
-        <is>
-          <t>COST DISTRIBUTION</t>
-        </is>
+          <t>Per Hour = Total Cost / Duration</t>
+        </is>
+      </c>
+      <c r="D30" s="12">
+        <f>D26/B4</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="6" t="inlineStr">
+        <is>
+          <t>Monthly projection (730 hrs always-on)</t>
+        </is>
+      </c>
+      <c r="D31" s="12">
+        <f>D30*730</f>
+        <v/>
       </c>
     </row>
     <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>Infrastructure (VM+Disk+SQL)</t>
-        </is>
-      </c>
-      <c r="C33" s="18">
-        <f>C16+C17+C18+C19</f>
-        <v/>
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>DEPLOY REGIONS:</t>
+        </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="19" t="inlineStr">
         <is>
-          <t>Microsoft Fabric (F2)</t>
-        </is>
-      </c>
-      <c r="C34" s="20">
-        <f>C20</f>
-        <v/>
+          <t>indonesiacentral</t>
+        </is>
+      </c>
+      <c r="B34" s="6" t="inlineStr">
+        <is>
+          <t>VM, Disk, SQL Hyperscale, Fabric F2, VNet, NSG</t>
+        </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>AI Tokens (GPT-5 + Embed)</t>
-        </is>
-      </c>
-      <c r="C35" s="18">
-        <f>C22+C23+C24</f>
-        <v/>
+      <c r="A35" s="19" t="inlineStr">
+        <is>
+          <t>eastus2</t>
+        </is>
+      </c>
+      <c r="B35" s="6" t="inlineStr">
+        <is>
+          <t>AI Foundry, GPT-5, text-embedding-3-small</t>
+        </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="21" t="inlineStr">
-        <is>
-          <t>TIP: Pause Fabric capacity &amp; deallocate VM when not in use to save $0.58/hr</t>
+      <c r="A37" s="20" t="inlineStr">
+        <is>
+          <t>DISCLAIMER:</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="21" t="inlineStr">
+        <is>
+          <t>Harga diperoleh melalui Azure Retail Prices API (https://prices.azure.com/api/retail/prices)</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="21" t="inlineStr">
+        <is>
+          <t>Harga dapat berubah sewaktu-waktu. Periksa Azure Portal untuk harga terkini.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="22" t="inlineStr">
+        <is>
+          <t>VM D2s_v5 Windows $0.200/hr SUDAH TERMASUK lisensi Windows Server.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="21" t="inlineStr">
+        <is>
+          <t>GPT-5: estimasi dari gpt-4o-1120 GlobalStandard (model belum tersedia di retail API).</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A1:F1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1704,16 +1805,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G12"/>
+  <dimension ref="A1:H14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="15" customWidth="1" min="1" max="1"/>
-    <col width="15" customWidth="1" min="2" max="2"/>
-    <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="15" customWidth="1" min="4" max="4"/>
-    <col width="15" customWidth="1" min="5" max="5"/>
-    <col width="15" customWidth="1" min="6" max="6"/>
-    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1724,264 +1826,308 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="9" t="inlineStr">
+      <c r="A3" s="10" t="inlineStr">
         <is>
           <t>Hour</t>
         </is>
       </c>
-      <c r="B3" s="9" t="inlineStr">
+      <c r="B3" s="10" t="inlineStr">
         <is>
           <t>VM ($)</t>
         </is>
       </c>
-      <c r="C3" s="9" t="inlineStr">
+      <c r="C3" s="10" t="inlineStr">
         <is>
           <t>Disk ($)</t>
         </is>
       </c>
-      <c r="D3" s="9" t="inlineStr">
+      <c r="D3" s="10" t="inlineStr">
         <is>
           <t>SQL ($)</t>
         </is>
       </c>
-      <c r="E3" s="9" t="inlineStr">
-        <is>
-          <t>Fabric F2 ($)</t>
-        </is>
-      </c>
-      <c r="F3" s="9" t="inlineStr">
+      <c r="E3" s="10" t="inlineStr">
+        <is>
+          <t>Fabric ($)</t>
+        </is>
+      </c>
+      <c r="F3" s="10" t="inlineStr">
         <is>
           <t>AI Tokens ($)</t>
         </is>
       </c>
-      <c r="G3" s="9" t="inlineStr">
+      <c r="G3" s="10" t="inlineStr">
+        <is>
+          <t>Hourly Total ($)</t>
+        </is>
+      </c>
+      <c r="H3" s="10" t="inlineStr">
         <is>
           <t>Running Total ($)</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="n">
+      <c r="A4" s="23" t="n">
         <v>1</v>
       </c>
-      <c r="B4" s="10" t="n">
+      <c r="B4" s="12" t="n">
         <v>0.2</v>
       </c>
-      <c r="C4" s="22">
+      <c r="C4" s="24">
         <f>5.89/730</f>
         <v/>
       </c>
-      <c r="D4" s="10" t="n">
+      <c r="D4" s="12" t="n">
         <v>0.6849</v>
       </c>
-      <c r="E4" s="13" t="n">
+      <c r="E4" s="15" t="n">
         <v>0.38</v>
       </c>
-      <c r="F4" s="22">
-        <f>(50*500/1000*0.0025 + 50*300/1000*0.01 + 100*200/1000*0.000025)/8</f>
-        <v/>
-      </c>
-      <c r="G4" s="23">
+      <c r="F4" s="24">
+        <f>(50*500/1000*0.0025+50*300/1000*0.01+100*200/1000*0.000025)/8</f>
+        <v/>
+      </c>
+      <c r="G4" s="12">
         <f>B4+C4+D4+E4+F4</f>
         <v/>
       </c>
+      <c r="H4" s="25">
+        <f>G4</f>
+        <v/>
+      </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="n">
+      <c r="A5" s="23" t="n">
         <v>2</v>
       </c>
-      <c r="B5" s="10" t="n">
+      <c r="B5" s="12" t="n">
         <v>0.2</v>
       </c>
-      <c r="C5" s="22">
+      <c r="C5" s="24">
         <f>5.89/730</f>
         <v/>
       </c>
-      <c r="D5" s="10" t="n">
+      <c r="D5" s="12" t="n">
         <v>0.6849</v>
       </c>
-      <c r="E5" s="13" t="n">
+      <c r="E5" s="15" t="n">
         <v>0.38</v>
       </c>
-      <c r="F5" s="22">
-        <f>(50*500/1000*0.0025 + 50*300/1000*0.01 + 100*200/1000*0.000025)/8</f>
-        <v/>
-      </c>
-      <c r="G5" s="23">
-        <f>G4+B5+C5+D5+E5+F5</f>
+      <c r="F5" s="24">
+        <f>(50*500/1000*0.0025+50*300/1000*0.01+100*200/1000*0.000025)/8</f>
+        <v/>
+      </c>
+      <c r="G5" s="12">
+        <f>B5+C5+D5+E5+F5</f>
+        <v/>
+      </c>
+      <c r="H5" s="25">
+        <f>H4+G5</f>
         <v/>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="n">
+      <c r="A6" s="23" t="n">
         <v>3</v>
       </c>
-      <c r="B6" s="10" t="n">
+      <c r="B6" s="12" t="n">
         <v>0.2</v>
       </c>
-      <c r="C6" s="22">
+      <c r="C6" s="24">
         <f>5.89/730</f>
         <v/>
       </c>
-      <c r="D6" s="10" t="n">
+      <c r="D6" s="12" t="n">
         <v>0.6849</v>
       </c>
-      <c r="E6" s="13" t="n">
+      <c r="E6" s="15" t="n">
         <v>0.38</v>
       </c>
-      <c r="F6" s="22">
-        <f>(50*500/1000*0.0025 + 50*300/1000*0.01 + 100*200/1000*0.000025)/8</f>
-        <v/>
-      </c>
-      <c r="G6" s="23">
-        <f>G5+B6+C6+D6+E6+F6</f>
+      <c r="F6" s="24">
+        <f>(50*500/1000*0.0025+50*300/1000*0.01+100*200/1000*0.000025)/8</f>
+        <v/>
+      </c>
+      <c r="G6" s="12">
+        <f>B6+C6+D6+E6+F6</f>
+        <v/>
+      </c>
+      <c r="H6" s="25">
+        <f>H5+G6</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="n">
+      <c r="A7" s="23" t="n">
         <v>4</v>
       </c>
-      <c r="B7" s="10" t="n">
+      <c r="B7" s="12" t="n">
         <v>0.2</v>
       </c>
-      <c r="C7" s="22">
+      <c r="C7" s="24">
         <f>5.89/730</f>
         <v/>
       </c>
-      <c r="D7" s="10" t="n">
+      <c r="D7" s="12" t="n">
         <v>0.6849</v>
       </c>
-      <c r="E7" s="13" t="n">
+      <c r="E7" s="15" t="n">
         <v>0.38</v>
       </c>
-      <c r="F7" s="22">
-        <f>(50*500/1000*0.0025 + 50*300/1000*0.01 + 100*200/1000*0.000025)/8</f>
-        <v/>
-      </c>
-      <c r="G7" s="23">
-        <f>G6+B7+C7+D7+E7+F7</f>
+      <c r="F7" s="24">
+        <f>(50*500/1000*0.0025+50*300/1000*0.01+100*200/1000*0.000025)/8</f>
+        <v/>
+      </c>
+      <c r="G7" s="12">
+        <f>B7+C7+D7+E7+F7</f>
+        <v/>
+      </c>
+      <c r="H7" s="25">
+        <f>H6+G7</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="n">
+      <c r="A8" s="23" t="n">
         <v>5</v>
       </c>
-      <c r="B8" s="10" t="n">
+      <c r="B8" s="12" t="n">
         <v>0.2</v>
       </c>
-      <c r="C8" s="22">
+      <c r="C8" s="24">
         <f>5.89/730</f>
         <v/>
       </c>
-      <c r="D8" s="10" t="n">
+      <c r="D8" s="12" t="n">
         <v>0.6849</v>
       </c>
-      <c r="E8" s="13" t="n">
+      <c r="E8" s="15" t="n">
         <v>0.38</v>
       </c>
-      <c r="F8" s="22">
-        <f>(50*500/1000*0.0025 + 50*300/1000*0.01 + 100*200/1000*0.000025)/8</f>
-        <v/>
-      </c>
-      <c r="G8" s="23">
-        <f>G7+B8+C8+D8+E8+F8</f>
+      <c r="F8" s="24">
+        <f>(50*500/1000*0.0025+50*300/1000*0.01+100*200/1000*0.000025)/8</f>
+        <v/>
+      </c>
+      <c r="G8" s="12">
+        <f>B8+C8+D8+E8+F8</f>
+        <v/>
+      </c>
+      <c r="H8" s="25">
+        <f>H7+G8</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="n">
+      <c r="A9" s="23" t="n">
         <v>6</v>
       </c>
-      <c r="B9" s="10" t="n">
+      <c r="B9" s="12" t="n">
         <v>0.2</v>
       </c>
-      <c r="C9" s="22">
+      <c r="C9" s="24">
         <f>5.89/730</f>
         <v/>
       </c>
-      <c r="D9" s="10" t="n">
+      <c r="D9" s="12" t="n">
         <v>0.6849</v>
       </c>
-      <c r="E9" s="13" t="n">
+      <c r="E9" s="15" t="n">
         <v>0.38</v>
       </c>
-      <c r="F9" s="22">
-        <f>(50*500/1000*0.0025 + 50*300/1000*0.01 + 100*200/1000*0.000025)/8</f>
-        <v/>
-      </c>
-      <c r="G9" s="23">
-        <f>G8+B9+C9+D9+E9+F9</f>
+      <c r="F9" s="24">
+        <f>(50*500/1000*0.0025+50*300/1000*0.01+100*200/1000*0.000025)/8</f>
+        <v/>
+      </c>
+      <c r="G9" s="12">
+        <f>B9+C9+D9+E9+F9</f>
+        <v/>
+      </c>
+      <c r="H9" s="25">
+        <f>H8+G9</f>
         <v/>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="n">
+      <c r="A10" s="23" t="n">
         <v>7</v>
       </c>
-      <c r="B10" s="10" t="n">
+      <c r="B10" s="12" t="n">
         <v>0.2</v>
       </c>
-      <c r="C10" s="22">
+      <c r="C10" s="24">
         <f>5.89/730</f>
         <v/>
       </c>
-      <c r="D10" s="10" t="n">
+      <c r="D10" s="12" t="n">
         <v>0.6849</v>
       </c>
-      <c r="E10" s="13" t="n">
+      <c r="E10" s="15" t="n">
         <v>0.38</v>
       </c>
-      <c r="F10" s="22">
-        <f>(50*500/1000*0.0025 + 50*300/1000*0.01 + 100*200/1000*0.000025)/8</f>
-        <v/>
-      </c>
-      <c r="G10" s="23">
-        <f>G9+B10+C10+D10+E10+F10</f>
+      <c r="F10" s="24">
+        <f>(50*500/1000*0.0025+50*300/1000*0.01+100*200/1000*0.000025)/8</f>
+        <v/>
+      </c>
+      <c r="G10" s="12">
+        <f>B10+C10+D10+E10+F10</f>
+        <v/>
+      </c>
+      <c r="H10" s="25">
+        <f>H9+G10</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="n">
+      <c r="A11" s="23" t="n">
         <v>8</v>
       </c>
-      <c r="B11" s="10" t="n">
+      <c r="B11" s="12" t="n">
         <v>0.2</v>
       </c>
-      <c r="C11" s="22">
+      <c r="C11" s="24">
         <f>5.89/730</f>
         <v/>
       </c>
-      <c r="D11" s="10" t="n">
+      <c r="D11" s="12" t="n">
         <v>0.6849</v>
       </c>
-      <c r="E11" s="13" t="n">
+      <c r="E11" s="15" t="n">
         <v>0.38</v>
       </c>
-      <c r="F11" s="22">
-        <f>(50*500/1000*0.0025 + 50*300/1000*0.01 + 100*200/1000*0.000025)/8</f>
-        <v/>
-      </c>
-      <c r="G11" s="23">
-        <f>G10+B11+C11+D11+E11+F11</f>
+      <c r="F11" s="24">
+        <f>(50*500/1000*0.0025+50*300/1000*0.01+100*200/1000*0.000025)/8</f>
+        <v/>
+      </c>
+      <c r="G11" s="12">
+        <f>B11+C11+D11+E11+F11</f>
+        <v/>
+      </c>
+      <c r="H11" s="25">
+        <f>H10+G11</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="24" t="inlineStr">
+      <c r="A12" s="26" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="G12" s="17">
-        <f>G11</f>
-        <v/>
+      <c r="H12" s="18">
+        <f>H11</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="8" t="inlineStr">
+        <is>
+          <t>Regions: VM/Disk/SQL/Fabric = indonesiacentral | AI Tokens = eastus2</t>
+        </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A1:H1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1993,13 +2139,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D22"/>
+  <dimension ref="A1:D18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="26" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="36" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="34" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2051,7 +2197,7 @@
           <t>F2 Hourly Cost</t>
         </is>
       </c>
-      <c r="B6" s="18">
+      <c r="B6" s="27">
         <f>2*0.19</f>
         <v/>
       </c>
@@ -2062,7 +2208,7 @@
           <t>F2 Monthly Cost (730hr)</t>
         </is>
       </c>
-      <c r="B7" s="18">
+      <c r="B7" s="27">
         <f>B6*730</f>
         <v/>
       </c>
@@ -2070,27 +2216,27 @@
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>FABRIC ITEMS IN LAB</t>
+          <t>FABRIC ITEMS</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="25" t="inlineStr">
+      <c r="A10" s="28" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
       </c>
-      <c r="B10" s="25" t="inlineStr">
+      <c r="B10" s="28" t="inlineStr">
         <is>
           <t>Type</t>
         </is>
       </c>
-      <c r="C10" s="25" t="inlineStr">
-        <is>
-          <t>CU Consumption</t>
-        </is>
-      </c>
-      <c r="D10" s="25" t="inlineStr">
+      <c r="C10" s="28" t="inlineStr">
+        <is>
+          <t>Region</t>
+        </is>
+      </c>
+      <c r="D10" s="28" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -2109,7 +2255,7 @@
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Container only</t>
+          <t>indonesiacentral</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
@@ -2131,7 +2277,7 @@
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Data Movement CUs</t>
+          <t>indonesiacentral</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
@@ -2148,12 +2294,12 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Auto-created endpoint</t>
+          <t>Auto-created</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Data Warehouse CUs</t>
+          <t>indonesiacentral</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
@@ -2175,12 +2321,12 @@
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Power BI CUs</t>
+          <t>indonesiacentral</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Storage mode: Direct Lake on SQL</t>
+          <t>Storage: Direct Lake on SQL</t>
         </is>
       </c>
     </row>
@@ -2197,7 +2343,7 @@
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Power BI CUs</t>
+          <t>indonesiacentral</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
@@ -2214,30 +2360,9 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="26" t="inlineStr">
-        <is>
-          <t>Azure SQL Hyperscale → Fabric Mirroring → OneLake (Delta) → SQL Endpoint → Semantic Model → Power BI</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="8" t="inlineStr">
-        <is>
-          <t>NOTE: All Fabric workloads consume CUs from the provisioned F2 capacity.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="8" t="inlineStr">
-        <is>
-          <t>No additional per-item cost beyond the F2 base rate of $0.38/hr.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="27" t="inlineStr">
-        <is>
-          <t>Pause capacity when not in use to stop billing.</t>
+      <c r="A18" s="29" t="inlineStr">
+        <is>
+          <t>Azure SQL Hyperscale -&gt; Fabric Mirroring -&gt; OneLake (Delta) -&gt; SQL Endpoint -&gt; Semantic Model -&gt; Power BI</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update SQL to Hyperscale Gen5 2-vCore (HS_S_Gen5_2), default 2 vCores
- SQL label: Hyperscale Gen5 Serverless (HS_S_Gen5_2)
- Default slider: 2.0 vCores (matches deploy.sh --capacity 2)
- Rate: -bash.6849/vCore/hr x 2 = .3698/hr at full utilization
- XLSX Sheet 2 updated with same
</commit_message>
<xml_diff>
--- a/cost-calculator-8hr.xlsx
+++ b/cost-calculator-8hr.xlsx
@@ -696,7 +696,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>HS_S_Gen5_2 Serverless</t>
+          <t>Hyperscale Gen5 Serverless (HS_S_Gen5_2)</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -722,7 +722,7 @@
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>Min 0.5, Max 2 vCores</t>
+          <t>2 vCores max; Serverless auto-pause</t>
         </is>
       </c>
     </row>
@@ -1304,11 +1304,11 @@
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
         <is>
-          <t>SQL vCore avg utilization</t>
+          <t>SQL vCores (Hyperscale Gen5)</t>
         </is>
       </c>
       <c r="B5" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
@@ -1317,7 +1317,7 @@
       </c>
       <c r="E5" s="8" t="inlineStr">
         <is>
-          <t>Range: 0.5 - 2.0</t>
+          <t>HS_S_Gen5_2 Serverless, max 2</t>
         </is>
       </c>
     </row>
@@ -1513,7 +1513,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>SQL Compute (Serverless Gen5)</t>
+          <t>SQL Hyperscale Gen5 (HS_S_Gen5_2)</t>
         </is>
       </c>
       <c r="B18" s="11" t="inlineStr">
@@ -1523,7 +1523,7 @@
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>8 hrs x vCores x $0.6849</t>
+          <t>8 hrs x 2 vCores x $0.6849</t>
         </is>
       </c>
       <c r="D18" s="12">

</xml_diff>